<commit_message>
Add dim_members with spec and tests
</commit_message>
<xml_diff>
--- a/docs/fact_dim_curation.xlsx
+++ b/docs/fact_dim_curation.xlsx
@@ -4,13 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12240" activeTab="3"/>
+    <workbookView windowWidth="28800" windowHeight="12240" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="fct_member_plan_month" sheetId="1" r:id="rId1"/>
     <sheet name="fct_member_month" sheetId="5" r:id="rId2"/>
     <sheet name="fct_medical_claim_lines" sheetId="7" r:id="rId3"/>
     <sheet name="singular_tests" sheetId="8" r:id="rId4"/>
+    <sheet name="dim_members" sheetId="10" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="345">
   <si>
     <t>Model Definition</t>
   </si>
@@ -988,6 +989,114 @@
   <si>
     <t>Equal start and end dates are valid; not_null checks are maintained in YAML.</t>
   </si>
+  <si>
+    <t>dim_members | Model Curation Specification</t>
+  </si>
+  <si>
+    <t>Grain: One row per member_id, including members without eligibility history</t>
+  </si>
+  <si>
+    <t>Latest = segment with greatest effective_date (tie-break: eligibility_segment_id descending); not current enrollment</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Source model</t>
+  </si>
+  <si>
+    <t>Transformation / rule</t>
+  </si>
+  <si>
+    <t>Nullable</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>stg_members</t>
+  </si>
+  <si>
+    <t>Unchanged</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Unique grain; retain all staged members</t>
+  </si>
+  <si>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>Synthetic member data</t>
+  </si>
+  <si>
+    <t>last_name</t>
+  </si>
+  <si>
+    <t>date_of_birth</t>
+  </si>
+  <si>
+    <t>Calculate age relative to reporting/service date downstream</t>
+  </si>
+  <si>
+    <t>gender_code</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>created_at</t>
+  </si>
+  <si>
+    <t>Source audit attribute</t>
+  </si>
+  <si>
+    <t>earliest_eligibility_effective_date</t>
+  </si>
+  <si>
+    <t>stg_eligibility_segments</t>
+  </si>
+  <si>
+    <t>min(effective_date) grouped by member_id</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Earliest date in available history, not necessarily first-ever enrollment</t>
+  </si>
+  <si>
+    <t>latest_eligibility_effective_date</t>
+  </si>
+  <si>
+    <t>effective_date from latest ranked segment</t>
+  </si>
+  <si>
+    <t>latest_eligibility_term_date</t>
+  </si>
+  <si>
+    <t>term_date from latest ranked segment</t>
+  </si>
+  <si>
+    <t>Also null when latest segment is open-ended</t>
+  </si>
+  <si>
+    <t>latest_plan_id</t>
+  </si>
+  <si>
+    <t>plan_id from latest ranked segment</t>
+  </si>
+  <si>
+    <t>Not necessarily a currently active plan</t>
+  </si>
+  <si>
+    <t>Implementation &amp; validation notes</t>
+  </si>
+  <si>
+    <t>Use a left join from stg_members to the one-row-per-member eligibility summary.</t>
+  </si>
 </sst>
 </file>
 
@@ -999,7 +1108,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1007,9 +1116,34 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <sz val="15"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF24476B"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF17365D"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -1036,13 +1170,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FF16324F"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -1059,7 +1186,8 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="18"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -1181,12 +1309,36 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="43">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF17365D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF1F8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2B557C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE8F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1197,12 +1349,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDCE8F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.05"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1558,139 +1704,163 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1698,55 +1868,52 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1758,40 +1925,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
@@ -2267,259 +2437,264 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="16.6666666666667" style="2" customWidth="1"/>
-    <col min="2" max="2" width="19.0092592592593" style="25" customWidth="1"/>
-    <col min="3" max="3" width="52.8333333333333" style="25" customWidth="1"/>
-    <col min="4" max="5" width="9.37037037037037" style="15" customWidth="1"/>
-    <col min="6" max="6" width="24.0648148148148" style="25" customWidth="1"/>
-    <col min="7" max="7" width="41.962962962963" style="25" customWidth="1"/>
-    <col min="8" max="8" width="25.5462962962963" style="25" customWidth="1"/>
-    <col min="9" max="16384" width="8.88888888888889" style="2"/>
+    <col min="1" max="1" width="19.0092592592593" style="32" customWidth="1"/>
+    <col min="2" max="2" width="52.8333333333333" style="32" customWidth="1"/>
+    <col min="3" max="4" width="9.37037037037037" style="22" customWidth="1"/>
+    <col min="5" max="5" width="24.0648148148148" style="32" customWidth="1"/>
+    <col min="6" max="6" width="41.962962962963" style="32" customWidth="1"/>
+    <col min="7" max="7" width="25.5462962962963" style="32" customWidth="1"/>
+    <col min="8" max="16384" width="8.88888888888889" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="23.4" spans="1:2">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="2:3">
-      <c r="B2" s="25" t="s">
+      <c r="B1" s="40"/>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="B2" s="32" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:3">
-      <c r="B3" s="25" t="s">
+    <row r="3" spans="1:2">
+      <c r="A3" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="B3" s="32" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:3">
-      <c r="B4" s="25" t="s">
+    <row r="4" spans="1:2">
+      <c r="A4" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="B4" s="32" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" ht="28.8" spans="2:4">
-      <c r="B5" s="25" t="s">
+    <row r="5" ht="28.8" spans="1:3">
+      <c r="A5" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="B5" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="25"/>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="2" t="s">
+      <c r="C5" s="32"/>
+    </row>
+    <row r="8" ht="23.4" spans="1:2">
+      <c r="A8" s="40" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="9" spans="2:8">
-      <c r="B9" s="33" t="s">
+      <c r="B8" s="40"/>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="B9" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="C9" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="33" t="s">
+      <c r="D9" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="33" t="s">
+      <c r="E9" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="33" t="s">
+      <c r="F9" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="33" t="s">
+      <c r="G9" s="41" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="2:6">
-      <c r="B10" s="25" t="s">
+    <row r="10" spans="1:5">
+      <c r="A10" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="B10" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="C10" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="D10" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="25" t="s">
+      <c r="E10" s="32" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="2:6">
-      <c r="B11" s="25" t="s">
+    <row r="11" spans="1:5">
+      <c r="A11" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="B11" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="C11" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="D11" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="E11" s="32" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="2:7">
-      <c r="B12" s="25" t="s">
+    <row r="12" spans="1:6">
+      <c r="A12" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="B12" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="C12" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="D12" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="F12" s="32" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="2:8">
-      <c r="B13" s="25" t="s">
+    <row r="13" spans="1:7">
+      <c r="A13" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="B13" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="D13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="F13" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="25" t="s">
+      <c r="G13" s="32" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="2:7">
-      <c r="B14" s="25" t="s">
+    <row r="14" spans="1:6">
+      <c r="A14" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="B14" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="D14" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="25" t="s">
+      <c r="F14" s="32" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" ht="28.8" spans="2:7">
-      <c r="B15" s="25" t="s">
+    <row r="15" ht="28.8" spans="1:6">
+      <c r="A15" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="B15" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="D15" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="25" t="s">
+      <c r="F15" s="32" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="2:7">
-      <c r="B16" s="25" t="s">
+    <row r="16" spans="1:6">
+      <c r="A16" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="B16" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="D16" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G16" s="25" t="s">
+      <c r="F16" s="32" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="17" spans="2:7">
-      <c r="B17" s="25" t="s">
+    <row r="17" spans="1:6">
+      <c r="A17" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="B17" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="D17" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="25" t="s">
+      <c r="F17" s="32" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="18" ht="28.8" spans="2:5">
-      <c r="B18" s="25" t="s">
+    <row r="18" ht="28.8" spans="1:4">
+      <c r="A18" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="B18" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="15" t="s">
+      <c r="D18" s="22" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" ht="43.2" spans="2:7">
-      <c r="B19" s="25" t="s">
+    <row r="19" ht="43.2" spans="1:6">
+      <c r="A19" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="B19" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="15" t="s">
+      <c r="D19" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="F19" s="32" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="2:3">
-      <c r="B21" s="34" t="s">
+    <row r="21" spans="1:2">
+      <c r="A21" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="B21" s="32" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="2:3">
-      <c r="B22" s="25" t="s">
+    <row r="22" spans="1:2">
+      <c r="A22" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="25" t="s">
+      <c r="B22" s="32" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="23" ht="28.8" spans="2:3">
-      <c r="B23" s="25" t="s">
+    <row r="23" ht="28.8" spans="1:2">
+      <c r="A23" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="25" t="s">
+      <c r="B23" s="32" t="s">
         <v>53</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A8:B8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
@@ -2531,485 +2706,485 @@
   <dimension ref="A1:H31"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="33.1111111111111" style="27" customWidth="1"/>
-    <col min="2" max="2" width="24.4444444444444" style="27" customWidth="1"/>
-    <col min="3" max="3" width="45.2222222222222" style="27" customWidth="1"/>
-    <col min="4" max="5" width="5.88888888888889" style="27" customWidth="1"/>
-    <col min="6" max="6" width="16.2222222222222" style="27" customWidth="1"/>
-    <col min="7" max="7" width="49.4444444444444" style="27" customWidth="1"/>
-    <col min="8" max="8" width="69.3333333333333" style="27" customWidth="1"/>
-    <col min="9" max="16384" width="10" style="27"/>
+    <col min="1" max="1" width="33.1111111111111" style="34" customWidth="1"/>
+    <col min="2" max="2" width="24.4444444444444" style="34" customWidth="1"/>
+    <col min="3" max="3" width="45.2222222222222" style="34" customWidth="1"/>
+    <col min="4" max="5" width="5.88888888888889" style="34" customWidth="1"/>
+    <col min="6" max="6" width="16.2222222222222" style="34" customWidth="1"/>
+    <col min="7" max="7" width="49.4444444444444" style="34" customWidth="1"/>
+    <col min="8" max="8" width="69.3333333333333" style="34" customWidth="1"/>
+    <col min="9" max="16384" width="10" style="34"/>
   </cols>
   <sheetData>
-    <row r="1" s="26" customFormat="1" ht="18" spans="1:8">
-      <c r="A1" s="13" t="s">
+    <row r="1" s="33" customFormat="1" ht="18" spans="1:8">
+      <c r="A1" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="34" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="34" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="34" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="34" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="34" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="8" ht="18" spans="1:8">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-    </row>
-    <row r="9" s="27" customFormat="1" ht="28.8" spans="1:8">
-      <c r="A9" s="18" t="s">
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+    </row>
+    <row r="9" s="34" customFormat="1" ht="28.8" spans="1:8">
+      <c r="A9" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="26" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" ht="28.8" spans="1:8">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="29" t="s">
+      <c r="D10" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="29" t="s">
+      <c r="E10" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="29" t="s">
+      <c r="F10" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="29" t="s">
+      <c r="G10" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="29" t="s">
+      <c r="H10" s="36" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="36" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="29" t="s">
+      <c r="D11" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="29" t="s">
+      <c r="E11" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29" t="s">
+      <c r="F11" s="36"/>
+      <c r="G11" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="H11" s="29" t="s">
+      <c r="H11" s="36" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29" t="s">
+      <c r="D12" s="36"/>
+      <c r="E12" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29" t="s">
+      <c r="F12" s="36"/>
+      <c r="G12" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="H12" s="29" t="s">
+      <c r="H12" s="36" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29" t="s">
+      <c r="D13" s="36"/>
+      <c r="E13" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29" t="s">
+      <c r="F13" s="36"/>
+      <c r="G13" s="36" t="s">
         <v>77</v>
       </c>
-      <c r="H13" s="29"/>
+      <c r="H13" s="36"/>
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:8">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="36" t="s">
         <v>79</v>
       </c>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29" t="s">
+      <c r="D14" s="36"/>
+      <c r="E14" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29" t="s">
+      <c r="F14" s="36"/>
+      <c r="G14" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="29" t="s">
+      <c r="H14" s="36" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="36" t="s">
         <v>81</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="C15" s="36" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29" t="s">
+      <c r="D15" s="36"/>
+      <c r="E15" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="29"/>
-      <c r="G15" s="29" t="s">
+      <c r="F15" s="36"/>
+      <c r="G15" s="36" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="29"/>
+      <c r="H15" s="36"/>
     </row>
     <row r="16" ht="28.8" spans="1:8">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29" t="s">
+      <c r="D16" s="36"/>
+      <c r="E16" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="29"/>
-      <c r="G16" s="29" t="s">
+      <c r="F16" s="36"/>
+      <c r="G16" s="36" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="29"/>
+      <c r="H16" s="36"/>
     </row>
     <row r="17" ht="26" customHeight="1" spans="1:8">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="36" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="36" t="s">
         <v>88</v>
       </c>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29" t="s">
+      <c r="D17" s="36"/>
+      <c r="E17" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="29"/>
-      <c r="G17" s="29" t="s">
+      <c r="F17" s="36"/>
+      <c r="G17" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="H17" s="29"/>
+      <c r="H17" s="36"/>
     </row>
     <row r="18" ht="43.2" spans="1:8">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="36" t="s">
         <v>91</v>
       </c>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29" t="s">
+      <c r="D18" s="36"/>
+      <c r="E18" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29" t="s">
+      <c r="F18" s="36"/>
+      <c r="G18" s="36" t="s">
         <v>93</v>
       </c>
-      <c r="H18" s="29" t="s">
+      <c r="H18" s="36" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:8">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="C19" s="36" t="s">
         <v>96</v>
       </c>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29" t="s">
+      <c r="D19" s="36"/>
+      <c r="E19" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="F19" s="29" t="s">
+      <c r="F19" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="29" t="s">
+      <c r="G19" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="H19" s="29" t="s">
+      <c r="H19" s="36" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="20" ht="28.8" spans="1:8">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29" t="s">
+      <c r="D20" s="36"/>
+      <c r="E20" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="F20" s="29"/>
-      <c r="G20" s="29" t="s">
+      <c r="F20" s="36"/>
+      <c r="G20" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="H20" s="29" t="s">
+      <c r="H20" s="36" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="21" ht="28.8" spans="1:8">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="29" t="s">
+      <c r="C21" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29" t="s">
+      <c r="D21" s="36"/>
+      <c r="E21" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="F21" s="29"/>
-      <c r="G21" s="29" t="s">
+      <c r="F21" s="36"/>
+      <c r="G21" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="H21" s="29" t="s">
+      <c r="H21" s="36" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="23" s="26" customFormat="1" ht="19" customHeight="1" spans="1:8">
-      <c r="A23" s="13" t="s">
+    <row r="23" s="33" customFormat="1" ht="19" customHeight="1" spans="1:8">
+      <c r="A23" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="B23" s="30" t="s">
+      <c r="B23" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="37"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
-      <c r="G24" s="31"/>
-      <c r="H24" s="31"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="38"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="38" t="s">
         <v>109</v>
       </c>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="38"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="36" t="s">
         <v>110</v>
       </c>
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="31"/>
-      <c r="H26" s="31"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="38"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="29" t="s">
+      <c r="A27" s="36" t="s">
         <v>112</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="31"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="36" t="s">
         <v>114</v>
       </c>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="38" t="s">
         <v>115</v>
       </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="31"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="36" t="s">
         <v>116</v>
       </c>
-      <c r="B29" s="31" t="s">
+      <c r="B29" s="38" t="s">
         <v>117</v>
       </c>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="31"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="38"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="32" t="s">
+      <c r="A30" s="39" t="s">
         <v>118</v>
       </c>
-      <c r="B30" s="31" t="s">
+      <c r="B30" s="38" t="s">
         <v>119</v>
       </c>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="31"/>
-      <c r="H30" s="31"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="32"/>
-      <c r="B31" s="32"/>
+      <c r="A31" s="39"/>
+      <c r="B31" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -3034,1067 +3209,1067 @@
   <dimension ref="A1:H55"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="23.7777777777778" style="11" customWidth="1"/>
-    <col min="2" max="2" width="28.2222222222222" style="2" customWidth="1"/>
-    <col min="3" max="3" width="11.2222222222222" style="2" customWidth="1"/>
-    <col min="4" max="4" width="39" style="2" customWidth="1"/>
-    <col min="5" max="6" width="9.88888888888889" style="2" customWidth="1"/>
-    <col min="7" max="7" width="29" style="2" customWidth="1"/>
-    <col min="8" max="8" width="80" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="8.88888888888889" style="2"/>
+    <col min="1" max="1" width="23.7777777777778" style="18" customWidth="1"/>
+    <col min="2" max="2" width="28.2222222222222" style="10" customWidth="1"/>
+    <col min="3" max="3" width="11.2222222222222" style="10" customWidth="1"/>
+    <col min="4" max="4" width="39" style="10" customWidth="1"/>
+    <col min="5" max="6" width="9.88888888888889" style="10" customWidth="1"/>
+    <col min="7" max="7" width="29" style="10" customWidth="1"/>
+    <col min="8" max="8" width="80" style="10" customWidth="1"/>
+    <col min="9" max="16384" width="8.88888888888889" style="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" ht="31" customHeight="1" spans="1:8">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
     </row>
     <row r="9" ht="25" customHeight="1" spans="1:8">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="25" t="s">
         <v>130</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="21">
+      <c r="A11" s="28">
         <v>1</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="29" t="s">
         <v>134</v>
       </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="21">
+      <c r="A12" s="28">
         <v>2</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="21">
+      <c r="A13" s="28">
         <v>3</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="21">
+      <c r="A14" s="28">
         <v>4</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="21">
+      <c r="A15" s="28">
         <v>5</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="C15" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="21">
+      <c r="A16" s="28">
         <v>6</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="29" t="s">
         <v>144</v>
       </c>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="21">
+      <c r="A17" s="28">
         <v>7</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="29" t="s">
         <v>146</v>
       </c>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="29"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="21">
+      <c r="A18" s="28">
         <v>8</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="29"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="21">
+      <c r="A19" s="28">
         <v>9</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="29" t="s">
         <v>150</v>
       </c>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="21"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
     </row>
     <row r="21" ht="25" customHeight="1" spans="1:8">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="B21" s="23"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="17"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="25" t="s">
         <v>151</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C22" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="D22" s="19" t="s">
+      <c r="D22" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="E22" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="H22" s="19" t="s">
+      <c r="H22" s="26" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="28" t="s">
         <v>133</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="27" t="s">
         <v>153</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="D23" s="27" t="s">
         <v>154</v>
       </c>
-      <c r="E23" s="20" t="s">
+      <c r="E23" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F23" s="20" t="s">
+      <c r="F23" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20" t="s">
+      <c r="G23" s="27"/>
+      <c r="H23" s="27" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="28" t="s">
         <v>133</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="27" t="s">
         <v>156</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="D24" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="E24" s="20" t="s">
+      <c r="E24" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F24" s="20" t="s">
+      <c r="F24" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20" t="s">
+      <c r="G24" s="27"/>
+      <c r="H24" s="27" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="27" t="s">
         <v>159</v>
       </c>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20" t="s">
+      <c r="E25" s="27"/>
+      <c r="F25" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G25" s="20" t="s">
+      <c r="G25" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="H25" s="20" t="s">
+      <c r="H25" s="27" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="C26" s="20" t="s">
+      <c r="C26" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="20" t="s">
+      <c r="D26" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20" t="s">
+      <c r="E26" s="27"/>
+      <c r="F26" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G26" s="24" t="s">
+      <c r="G26" s="31" t="s">
         <v>163</v>
       </c>
-      <c r="H26" s="20" t="s">
+      <c r="H26" s="27" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="C27" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="20" t="s">
+      <c r="D27" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20" t="s">
+      <c r="E27" s="27"/>
+      <c r="F27" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G27" s="20" t="s">
+      <c r="G27" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="H27" s="20" t="s">
+      <c r="H27" s="27" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="28" ht="28.8" spans="1:8">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="27" t="s">
         <v>166</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="C28" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="D28" s="20" t="s">
+      <c r="D28" s="27" t="s">
         <v>167</v>
       </c>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20" t="s">
+      <c r="E28" s="27"/>
+      <c r="F28" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20" t="s">
+      <c r="G28" s="27"/>
+      <c r="H28" s="27" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="21" t="s">
+      <c r="A29" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="27" t="s">
         <v>169</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="D29" s="27" t="s">
         <v>170</v>
       </c>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20" t="s">
+      <c r="E29" s="27"/>
+      <c r="F29" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G29" s="20"/>
-      <c r="H29" s="20" t="s">
+      <c r="G29" s="27"/>
+      <c r="H29" s="27" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="21" t="s">
+      <c r="A30" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="27" t="s">
         <v>172</v>
       </c>
-      <c r="C30" s="20" t="s">
+      <c r="C30" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="20" t="s">
+      <c r="D30" s="27" t="s">
         <v>173</v>
       </c>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20" t="s">
+      <c r="E30" s="27"/>
+      <c r="F30" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G30" s="20"/>
-      <c r="H30" s="20" t="s">
+      <c r="G30" s="27"/>
+      <c r="H30" s="27" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="B31" s="20" t="s">
+      <c r="B31" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="C31" s="20" t="s">
+      <c r="C31" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="27" t="s">
         <v>176</v>
       </c>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20" t="s">
+      <c r="E31" s="27"/>
+      <c r="F31" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G31" s="20"/>
-      <c r="H31" s="20" t="s">
+      <c r="G31" s="27"/>
+      <c r="H31" s="27" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="27" t="s">
         <v>177</v>
       </c>
-      <c r="C32" s="20" t="s">
+      <c r="C32" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="D32" s="27" t="s">
         <v>178</v>
       </c>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20" t="s">
+      <c r="E32" s="27"/>
+      <c r="F32" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G32" s="20"/>
-      <c r="H32" s="20" t="s">
+      <c r="G32" s="27"/>
+      <c r="H32" s="27" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="21" t="s">
+      <c r="A33" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="27" t="s">
         <v>180</v>
       </c>
-      <c r="C33" s="20" t="s">
+      <c r="C33" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D33" s="20" t="s">
+      <c r="D33" s="27" t="s">
         <v>181</v>
       </c>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20" t="s">
+      <c r="E33" s="27"/>
+      <c r="F33" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20" t="s">
+      <c r="G33" s="27"/>
+      <c r="H33" s="27" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:8">
-      <c r="A34" s="21" t="s">
+      <c r="A34" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="20" t="s">
+      <c r="B34" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="C34" s="20" t="s">
+      <c r="C34" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="D34" s="20" t="s">
+      <c r="D34" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20" t="s">
+      <c r="E34" s="27"/>
+      <c r="F34" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20" t="s">
+      <c r="G34" s="27"/>
+      <c r="H34" s="27" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1" spans="1:8">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="B35" s="20" t="s">
+      <c r="B35" s="27" t="s">
         <v>186</v>
       </c>
-      <c r="C35" s="20" t="s">
+      <c r="C35" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="D35" s="25" t="s">
+      <c r="D35" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E35" s="35" t="s">
+      <c r="E35" s="43" t="s">
         <v>188</v>
       </c>
-      <c r="F35" s="20" t="s">
+      <c r="F35" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20" t="s">
+      <c r="G35" s="27"/>
+      <c r="H35" s="27" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:8">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="B36" s="20" t="s">
+      <c r="B36" s="27" t="s">
         <v>190</v>
       </c>
-      <c r="C36" s="20" t="s">
+      <c r="C36" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="D36" s="20" t="s">
+      <c r="D36" s="27" t="s">
         <v>191</v>
       </c>
-      <c r="E36" s="20"/>
-      <c r="F36" s="20" t="s">
+      <c r="E36" s="27"/>
+      <c r="F36" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20" t="s">
+      <c r="G36" s="27"/>
+      <c r="H36" s="27" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="37" spans="1:8">
-      <c r="A37" s="21" t="s">
+      <c r="A37" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="B37" s="20" t="s">
+      <c r="B37" s="27" t="s">
         <v>193</v>
       </c>
-      <c r="C37" s="20" t="s">
+      <c r="C37" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="D37" s="20" t="s">
+      <c r="D37" s="27" t="s">
         <v>194</v>
       </c>
-      <c r="E37" s="20"/>
-      <c r="F37" s="20" t="s">
+      <c r="E37" s="27"/>
+      <c r="F37" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G37" s="20"/>
-      <c r="H37" s="20" t="s">
+      <c r="G37" s="27"/>
+      <c r="H37" s="27" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="38" spans="1:8">
-      <c r="A38" s="21" t="s">
+      <c r="A38" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="B38" s="20" t="s">
+      <c r="B38" s="27" t="s">
         <v>196</v>
       </c>
-      <c r="C38" s="20" t="s">
+      <c r="C38" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="D38" s="20" t="s">
+      <c r="D38" s="27" t="s">
         <v>197</v>
       </c>
-      <c r="E38" s="20"/>
-      <c r="F38" s="20" t="s">
+      <c r="E38" s="27"/>
+      <c r="F38" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G38" s="20"/>
-      <c r="H38" s="20" t="s">
+      <c r="G38" s="27"/>
+      <c r="H38" s="27" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:8">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="B39" s="20" t="s">
+      <c r="B39" s="27" t="s">
         <v>199</v>
       </c>
-      <c r="C39" s="20" t="s">
+      <c r="C39" s="27" t="s">
         <v>200</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D39" s="27" t="s">
         <v>201</v>
       </c>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20" t="s">
+      <c r="E39" s="27"/>
+      <c r="F39" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20" t="s">
+      <c r="G39" s="27"/>
+      <c r="H39" s="27" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="40" ht="28.8" spans="1:8">
-      <c r="A40" s="21" t="s">
+      <c r="A40" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="B40" s="20" t="s">
+      <c r="B40" s="27" t="s">
         <v>203</v>
       </c>
-      <c r="C40" s="20" t="s">
+      <c r="C40" s="27" t="s">
         <v>204</v>
       </c>
-      <c r="D40" s="20" t="s">
+      <c r="D40" s="27" t="s">
         <v>205</v>
       </c>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20" t="s">
+      <c r="E40" s="27"/>
+      <c r="F40" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20" t="s">
+      <c r="G40" s="27"/>
+      <c r="H40" s="27" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="41" ht="28.8" spans="1:8">
-      <c r="A41" s="21" t="s">
+      <c r="A41" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="B41" s="20" t="s">
+      <c r="B41" s="27" t="s">
         <v>207</v>
       </c>
-      <c r="C41" s="20" t="s">
+      <c r="C41" s="27" t="s">
         <v>204</v>
       </c>
-      <c r="D41" s="20" t="s">
+      <c r="D41" s="27" t="s">
         <v>208</v>
       </c>
-      <c r="E41" s="20"/>
-      <c r="F41" s="20" t="s">
+      <c r="E41" s="27"/>
+      <c r="F41" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G41" s="20"/>
-      <c r="H41" s="20" t="s">
+      <c r="G41" s="27"/>
+      <c r="H41" s="27" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="42" ht="28.8" spans="1:8">
-      <c r="A42" s="21" t="s">
+      <c r="A42" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="B42" s="20" t="s">
+      <c r="B42" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="C42" s="20" t="s">
+      <c r="C42" s="27" t="s">
         <v>204</v>
       </c>
-      <c r="D42" s="20" t="s">
+      <c r="D42" s="27" t="s">
         <v>210</v>
       </c>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20" t="s">
+      <c r="E42" s="27"/>
+      <c r="F42" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G42" s="20"/>
-      <c r="H42" s="20" t="s">
+      <c r="G42" s="27"/>
+      <c r="H42" s="27" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="43" ht="28.8" spans="1:8">
-      <c r="A43" s="21" t="s">
+      <c r="A43" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="B43" s="20" t="s">
+      <c r="B43" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="C43" s="20" t="s">
+      <c r="C43" s="27" t="s">
         <v>204</v>
       </c>
-      <c r="D43" s="20" t="s">
+      <c r="D43" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20" t="s">
+      <c r="E43" s="27"/>
+      <c r="F43" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G43" s="20"/>
-      <c r="H43" s="20" t="s">
+      <c r="G43" s="27"/>
+      <c r="H43" s="27" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="44" spans="1:8">
-      <c r="A44" s="21" t="s">
+      <c r="A44" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="B44" s="20" t="s">
+      <c r="B44" s="27" t="s">
         <v>213</v>
       </c>
-      <c r="C44" s="20" t="s">
+      <c r="C44" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="20" t="s">
+      <c r="D44" s="27" t="s">
         <v>214</v>
       </c>
-      <c r="E44" s="20"/>
-      <c r="F44" s="20" t="s">
+      <c r="E44" s="27"/>
+      <c r="F44" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G44" s="20"/>
-      <c r="H44" s="20" t="s">
+      <c r="G44" s="27"/>
+      <c r="H44" s="27" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="45" spans="1:8">
-      <c r="A45" s="21" t="s">
+      <c r="A45" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="B45" s="20" t="s">
+      <c r="B45" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="C45" s="20" t="s">
+      <c r="C45" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D45" s="20" t="s">
+      <c r="D45" s="27" t="s">
         <v>217</v>
       </c>
-      <c r="E45" s="20"/>
-      <c r="F45" s="20" t="s">
+      <c r="E45" s="27"/>
+      <c r="F45" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G45" s="20"/>
-      <c r="H45" s="20" t="s">
+      <c r="G45" s="27"/>
+      <c r="H45" s="27" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="46" spans="1:8">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="B46" s="20" t="s">
+      <c r="B46" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="C46" s="20" t="s">
+      <c r="C46" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D46" s="20" t="s">
+      <c r="D46" s="27" t="s">
         <v>219</v>
       </c>
-      <c r="E46" s="20"/>
-      <c r="F46" s="20" t="s">
+      <c r="E46" s="27"/>
+      <c r="F46" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G46" s="20"/>
-      <c r="H46" s="20" t="s">
+      <c r="G46" s="27"/>
+      <c r="H46" s="27" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="47" spans="1:8">
-      <c r="A47" s="21" t="s">
+      <c r="A47" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="B47" s="20" t="s">
+      <c r="B47" s="27" t="s">
         <v>221</v>
       </c>
-      <c r="C47" s="20" t="s">
+      <c r="C47" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D47" s="20" t="s">
+      <c r="D47" s="27" t="s">
         <v>222</v>
       </c>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20" t="s">
+      <c r="E47" s="27"/>
+      <c r="F47" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G47" s="20"/>
-      <c r="H47" s="20" t="s">
+      <c r="G47" s="27"/>
+      <c r="H47" s="27" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="48" spans="1:8">
-      <c r="A48" s="21" t="s">
+      <c r="A48" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="B48" s="20" t="s">
+      <c r="B48" s="27" t="s">
         <v>224</v>
       </c>
-      <c r="C48" s="20" t="s">
+      <c r="C48" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D48" s="20" t="s">
+      <c r="D48" s="27" t="s">
         <v>225</v>
       </c>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20" t="s">
+      <c r="E48" s="27"/>
+      <c r="F48" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G48" s="20"/>
-      <c r="H48" s="20" t="s">
+      <c r="G48" s="27"/>
+      <c r="H48" s="27" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="49" spans="1:8">
-      <c r="A49" s="21" t="s">
+      <c r="A49" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="B49" s="20" t="s">
+      <c r="B49" s="27" t="s">
         <v>226</v>
       </c>
-      <c r="C49" s="20" t="s">
+      <c r="C49" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D49" s="20" t="s">
+      <c r="D49" s="27" t="s">
         <v>227</v>
       </c>
-      <c r="E49" s="20"/>
-      <c r="F49" s="20" t="s">
+      <c r="E49" s="27"/>
+      <c r="F49" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G49" s="20"/>
-      <c r="H49" s="20" t="s">
+      <c r="G49" s="27"/>
+      <c r="H49" s="27" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="50" spans="1:8">
-      <c r="A50" s="21" t="s">
+      <c r="A50" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="B50" s="20" t="s">
+      <c r="B50" s="27" t="s">
         <v>228</v>
       </c>
-      <c r="C50" s="20" t="s">
+      <c r="C50" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D50" s="20" t="s">
+      <c r="D50" s="27" t="s">
         <v>229</v>
       </c>
-      <c r="E50" s="20"/>
-      <c r="F50" s="20" t="s">
+      <c r="E50" s="27"/>
+      <c r="F50" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G50" s="20"/>
-      <c r="H50" s="20" t="s">
+      <c r="G50" s="27"/>
+      <c r="H50" s="27" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="51" spans="1:8">
-      <c r="A51" s="21" t="s">
+      <c r="A51" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="B51" s="20" t="s">
+      <c r="B51" s="27" t="s">
         <v>230</v>
       </c>
-      <c r="C51" s="20" t="s">
+      <c r="C51" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D51" s="20" t="s">
+      <c r="D51" s="27" t="s">
         <v>231</v>
       </c>
-      <c r="E51" s="20"/>
-      <c r="F51" s="20" t="s">
+      <c r="E51" s="27"/>
+      <c r="F51" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20" t="s">
+      <c r="G51" s="27"/>
+      <c r="H51" s="27" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="52" spans="1:8">
-      <c r="A52" s="21" t="s">
+      <c r="A52" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="B52" s="20" t="s">
+      <c r="B52" s="27" t="s">
         <v>233</v>
       </c>
-      <c r="C52" s="20" t="s">
+      <c r="C52" s="27" t="s">
         <v>234</v>
       </c>
-      <c r="D52" s="20" t="s">
+      <c r="D52" s="27" t="s">
         <v>235</v>
       </c>
-      <c r="E52" s="20"/>
-      <c r="F52" s="20" t="s">
+      <c r="E52" s="27"/>
+      <c r="F52" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20" t="s">
+      <c r="G52" s="27"/>
+      <c r="H52" s="27" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="53" spans="1:8">
-      <c r="A53" s="21" t="s">
+      <c r="A53" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="B53" s="20" t="s">
+      <c r="B53" s="27" t="s">
         <v>237</v>
       </c>
-      <c r="C53" s="20" t="s">
+      <c r="C53" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D53" s="20" t="s">
+      <c r="D53" s="27" t="s">
         <v>238</v>
       </c>
-      <c r="E53" s="20"/>
-      <c r="F53" s="20" t="s">
+      <c r="E53" s="27"/>
+      <c r="F53" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G53" s="20"/>
-      <c r="H53" s="20" t="s">
+      <c r="G53" s="27"/>
+      <c r="H53" s="27" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="54" spans="1:8">
-      <c r="A54" s="21" t="s">
+      <c r="A54" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="B54" s="20" t="s">
+      <c r="B54" s="27" t="s">
         <v>240</v>
       </c>
-      <c r="C54" s="20" t="s">
+      <c r="C54" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D54" s="20" t="s">
+      <c r="D54" s="27" t="s">
         <v>241</v>
       </c>
-      <c r="E54" s="20"/>
-      <c r="F54" s="20" t="s">
+      <c r="E54" s="27"/>
+      <c r="F54" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20" t="s">
+      <c r="G54" s="27"/>
+      <c r="H54" s="27" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="55" spans="1:8">
-      <c r="A55" s="21" t="s">
+      <c r="A55" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="B55" s="20" t="s">
+      <c r="B55" s="27" t="s">
         <v>242</v>
       </c>
-      <c r="C55" s="20" t="s">
+      <c r="C55" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D55" s="20" t="s">
+      <c r="D55" s="27" t="s">
         <v>243</v>
       </c>
-      <c r="E55" s="20"/>
-      <c r="F55" s="20" t="s">
+      <c r="E55" s="27"/>
+      <c r="F55" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="G55" s="20"/>
-      <c r="H55" s="20" t="s">
+      <c r="G55" s="27"/>
+      <c r="H55" s="27" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4129,346 +4304,346 @@
   <dimension ref="A1:I12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="49.1111111111111" style="2" customWidth="1"/>
-    <col min="2" max="2" width="34.8888888888889" style="2" customWidth="1"/>
-    <col min="3" max="3" width="29" style="2" customWidth="1"/>
-    <col min="4" max="4" width="52.4444444444444" style="2" customWidth="1"/>
-    <col min="5" max="6" width="40" style="2" customWidth="1"/>
-    <col min="7" max="7" width="8" style="2" customWidth="1"/>
-    <col min="8" max="8" width="7.44444444444444" style="2" customWidth="1"/>
-    <col min="9" max="9" width="21.5555555555556" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="2"/>
+    <col min="1" max="1" width="49.1111111111111" style="10" customWidth="1"/>
+    <col min="2" max="2" width="34.8888888888889" style="10" customWidth="1"/>
+    <col min="3" max="3" width="29" style="10" customWidth="1"/>
+    <col min="4" max="4" width="52.4444444444444" style="10" customWidth="1"/>
+    <col min="5" max="6" width="40" style="10" customWidth="1"/>
+    <col min="7" max="7" width="8" style="10" customWidth="1"/>
+    <col min="8" max="8" width="7.44444444444444" style="10" customWidth="1"/>
+    <col min="9" max="9" width="21.5555555555556" style="10" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:9">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" ht="27" customHeight="1" spans="1:9">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="12" t="s">
         <v>250</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="12" t="s">
         <v>251</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="15" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A3" s="5" t="s">
+    <row r="3" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A3" s="13" t="s">
         <v>254</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="13" t="s">
         <v>255</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="13" t="s">
         <v>257</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="13" t="s">
         <v>258</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="16" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A4" s="5" t="s">
+    <row r="4" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A4" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="13" t="s">
         <v>264</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="13" t="s">
         <v>265</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="16" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A5" s="5" t="s">
+    <row r="5" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A5" s="13" t="s">
         <v>267</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="13" t="s">
         <v>268</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="13" t="s">
         <v>269</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="13" t="s">
         <v>270</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="13" t="s">
         <v>271</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="16" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A6" s="5" t="s">
+    <row r="6" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A6" s="13" t="s">
         <v>272</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="13" t="s">
         <v>273</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="13" t="s">
         <v>274</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="13" t="s">
         <v>275</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="13" t="s">
         <v>276</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="16" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A7" s="5" t="s">
+    <row r="7" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A7" s="13" t="s">
         <v>277</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="13" t="s">
         <v>278</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="13" t="s">
         <v>279</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="13" t="s">
         <v>280</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="13" t="s">
         <v>281</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="16" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A8" s="6" t="s">
+    <row r="8" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A8" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>286</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="14" t="s">
         <v>260</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="17" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A9" s="6" t="s">
+    <row r="9" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A9" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="14" t="s">
         <v>260</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="17" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A10" s="6" t="s">
+    <row r="10" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A10" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>294</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="17" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A11" s="6" t="s">
+    <row r="11" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A11" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="14" t="s">
         <v>301</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="14" t="s">
         <v>302</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="14" t="s">
         <v>303</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="17" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A12" s="6" t="s">
+    <row r="12" s="9" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A12" s="14" t="s">
         <v>304</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="14" t="s">
         <v>305</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="14" t="s">
         <v>307</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="14" t="s">
         <v>308</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="17" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4476,4 +4651,293 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="31.6666666666667" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.8888888888889" style="1" customWidth="1"/>
+    <col min="3" max="3" width="42.3333333333333" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.4444444444444" style="1" customWidth="1"/>
+    <col min="5" max="5" width="63" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="10" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:5">
+      <c r="A1" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" spans="1:5">
+      <c r="A19" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="8" t="s">
+        <v>344</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A20:E20"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>